<commit_message>
Add card, cards, product-filters blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (7):
- blocks/card/card.js
- blocks/cards/cards.js
- blocks/product-filters/product-filters.js
- tools/importer/import-portfolio-category.bundle.js
- tools/importer/parsers/cards.js
- tools/importer/reports/import-portfolio-category.report.xlsx
- tools/importer/reports/us/en/portfolios/medical-surgical-equipment/bedframes.report.json
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-portfolio-category.report.xlsx
+++ b/tools/importer/reports/import-portfolio-category.report.xlsx
@@ -40,7 +40,7 @@
     <t>us/en/portfolios/medical-surgical-equipment/bedframes.report.json</t>
   </si>
   <si>
-    <t>["hero","cards","cards","columns"]</t>
+    <t>["hero","cards","cards","product-filters","columns"]</t>
   </si>
   <si>
     <t>us/en/portfolios/medical-surgical-equipment/bedframes</t>
@@ -52,7 +52,7 @@
     <t>portfolio-category</t>
   </si>
   <si>
-    <t>2026-04-21T20:50:17.531Z</t>
+    <t>2026-04-25T14:53:31.277Z</t>
   </si>
   <si>
     <t>Bed frames | Stryker</t>
@@ -450,9 +450,7 @@
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="50" customWidth="1"/>
-    <col min="2" max="2" width="36" customWidth="1"/>
-    <col min="3" max="3" width="50" customWidth="1"/>
+    <col min="1" max="3" width="50" customWidth="1"/>
     <col min="5" max="5" width="20" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
     <col min="7" max="7" width="22" customWidth="1"/>

</xml_diff>